<commit_message>
Momentum scan results 2026-09-29
</commit_message>
<xml_diff>
--- a/results/momentum_2026-09-29.xlsx
+++ b/results/momentum_2026-09-29.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,146 +441,46 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>ASST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>ABCL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CAI</t>
+          <t>IOVA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>KLAC</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>AMKR</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>CBRS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>IOVA</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ISRG</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>QMCO</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>NTAP</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>PLTR</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>MXL</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TEM</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>SDGR</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>QUBT</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>USDE</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>STRC</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>OUST</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>MRNA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>SECZ</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>ILMN</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>GLND</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
+          <t>COIN</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>